<commit_message>
Fixed indexing in script to input BAU capacities and costs, updated BAU capacities for PV and wind for milestone II countries
</commit_message>
<xml_diff>
--- a/Code/format_weather_profiles/onshorebau_max_cap_calc.xlsx
+++ b/Code/format_weather_profiles/onshorebau_max_cap_calc.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/laorie4253/Documents/MOYA Analytics/GMPA/STEVFNs/Code/format_weather_profiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{ED1C0E3F-09A0-304D-8A62-DDDF4CE98B0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3480195D-C7CB-4045-8F12-BA48107C66D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="1240" windowWidth="27640" windowHeight="16760" xr2:uid="{0A39901E-EE16-E845-B782-0D9319A9913F}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="27640" windowHeight="16760" xr2:uid="{0A39901E-EE16-E845-B782-0D9319A9913F}"/>
   </bookViews>
   <sheets>
     <sheet name="onshorebau_max_cap" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -181,7 +181,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -212,6 +212,24 @@
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -225,7 +243,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -245,6 +263,18 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1263,174 +1293,186 @@
       <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B12" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C12" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D12" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E12" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F12" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G12" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H12" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I12" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J12" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K12" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L12" t="e">
-        <f t="shared" si="10"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M12" s="4">
-        <v>11.327</v>
-      </c>
-      <c r="N12" s="7"/>
-      <c r="O12" s="7"/>
-      <c r="P12" t="e">
-        <f t="shared" si="11"/>
-        <v>#DIV/0!</v>
+      <c r="B12">
+        <f t="shared" si="0"/>
+        <v>0.67927177766812219</v>
+      </c>
+      <c r="C12">
+        <f t="shared" si="1"/>
+        <v>0.67927177766812219</v>
+      </c>
+      <c r="D12">
+        <f t="shared" si="2"/>
+        <v>0.67927177766812219</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="3"/>
+        <v>0.67927177766812219</v>
+      </c>
+      <c r="F12">
+        <f t="shared" si="4"/>
+        <v>0.67927177766812219</v>
+      </c>
+      <c r="G12">
+        <f t="shared" si="5"/>
+        <v>0.67927177766812219</v>
+      </c>
+      <c r="H12">
+        <f t="shared" si="6"/>
+        <v>0.67927177766812219</v>
+      </c>
+      <c r="I12">
+        <f t="shared" si="7"/>
+        <v>0.67927177766812219</v>
+      </c>
+      <c r="J12">
+        <f t="shared" si="8"/>
+        <v>0.67927177766812219</v>
+      </c>
+      <c r="K12">
+        <f t="shared" si="9"/>
+        <v>0.67927177766812219</v>
+      </c>
+      <c r="L12">
+        <f t="shared" si="10"/>
+        <v>6.7927177766812221</v>
+      </c>
+      <c r="M12" s="9">
+        <v>4.181</v>
+      </c>
+      <c r="N12">
+        <v>252359.96200000035</v>
+      </c>
+      <c r="O12">
+        <v>410000</v>
+      </c>
+      <c r="P12">
+        <f t="shared" si="11"/>
+        <v>1.6246634242241622</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B13" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C13" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D13" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E13" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F13" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G13" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H13" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I13" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J13" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K13" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L13" t="e">
-        <f t="shared" si="10"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M13" s="2">
-        <v>0.40300000000000002</v>
-      </c>
-      <c r="N13" s="7"/>
-      <c r="O13" s="7"/>
-      <c r="P13" t="e">
-        <f t="shared" si="11"/>
-        <v>#DIV/0!</v>
+      <c r="B13">
+        <f t="shared" si="0"/>
+        <v>2.252105874157106E-4</v>
+      </c>
+      <c r="C13">
+        <f t="shared" si="1"/>
+        <v>2.252105874157106E-4</v>
+      </c>
+      <c r="D13">
+        <f t="shared" si="2"/>
+        <v>2.252105874157106E-4</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="3"/>
+        <v>2.252105874157106E-4</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="4"/>
+        <v>2.252105874157106E-4</v>
+      </c>
+      <c r="G13">
+        <f t="shared" si="5"/>
+        <v>2.252105874157106E-4</v>
+      </c>
+      <c r="H13">
+        <f t="shared" si="6"/>
+        <v>2.252105874157106E-4</v>
+      </c>
+      <c r="I13">
+        <f t="shared" si="7"/>
+        <v>2.252105874157106E-4</v>
+      </c>
+      <c r="J13">
+        <f t="shared" si="8"/>
+        <v>2.252105874157106E-4</v>
+      </c>
+      <c r="K13">
+        <f t="shared" si="9"/>
+        <v>2.252105874157106E-4</v>
+      </c>
+      <c r="L13">
+        <f t="shared" si="10"/>
+        <v>2.252105874157106E-3</v>
+      </c>
+      <c r="M13" s="10">
+        <v>1E-3</v>
+      </c>
+      <c r="N13">
+        <v>338349.99000000086</v>
+      </c>
+      <c r="O13">
+        <v>762000</v>
+      </c>
+      <c r="P13">
+        <f t="shared" si="11"/>
+        <v>2.2521058741571061</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B14" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C14" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D14" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E14" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F14" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G14" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H14" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I14" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J14" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K14" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L14" t="e">
-        <f t="shared" si="10"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M14" s="4">
-        <v>44.735999999999997</v>
-      </c>
-      <c r="N14" s="7"/>
-      <c r="O14" s="7"/>
-      <c r="P14" t="e">
-        <f t="shared" si="11"/>
-        <v>#DIV/0!</v>
+      <c r="B14">
+        <f t="shared" si="0"/>
+        <v>6.7530869924559722</v>
+      </c>
+      <c r="C14">
+        <f t="shared" si="1"/>
+        <v>6.7530869924559722</v>
+      </c>
+      <c r="D14">
+        <f t="shared" si="2"/>
+        <v>6.7530869924559722</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="3"/>
+        <v>6.7530869924559722</v>
+      </c>
+      <c r="F14">
+        <f t="shared" si="4"/>
+        <v>6.7530869924559722</v>
+      </c>
+      <c r="G14">
+        <f t="shared" si="5"/>
+        <v>6.7530869924559722</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="6"/>
+        <v>6.7530869924559722</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="7"/>
+        <v>6.7530869924559722</v>
+      </c>
+      <c r="J14">
+        <f t="shared" si="8"/>
+        <v>6.7530869924559722</v>
+      </c>
+      <c r="K14">
+        <f t="shared" si="9"/>
+        <v>6.7530869924559722</v>
+      </c>
+      <c r="L14">
+        <f t="shared" si="10"/>
+        <v>67.530869924559724</v>
+      </c>
+      <c r="M14" s="11">
+        <v>25.088000000000001</v>
+      </c>
+      <c r="N14">
+        <v>1383110.0370000005</v>
+      </c>
+      <c r="O14">
+        <v>3723000</v>
+      </c>
+      <c r="P14">
+        <f t="shared" si="11"/>
+        <v>2.6917598024776672</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
@@ -1481,11 +1523,9 @@
         <f t="shared" si="10"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="M15" s="5">
+      <c r="M15" s="9">
         <v>0.104</v>
       </c>
-      <c r="N15" s="7"/>
-      <c r="O15" s="7"/>
       <c r="P15" t="e">
         <f t="shared" si="11"/>
         <v>#DIV/0!</v>
@@ -2115,371 +2155,434 @@
       <c r="A26" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B26" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C26" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D26" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E26" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F26" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G26" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H26" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I26" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J26" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K26" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L26" t="e">
-        <f t="shared" si="10"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P26" t="e">
-        <f t="shared" si="11"/>
-        <v>#DIV/0!</v>
+      <c r="B26">
+        <f t="shared" si="0"/>
+        <v>1.4115708063811312</v>
+      </c>
+      <c r="C26">
+        <f t="shared" si="1"/>
+        <v>1.4115708063811312</v>
+      </c>
+      <c r="D26">
+        <f t="shared" si="2"/>
+        <v>1.4115708063811312</v>
+      </c>
+      <c r="E26">
+        <f t="shared" si="3"/>
+        <v>1.4115708063811312</v>
+      </c>
+      <c r="F26">
+        <f t="shared" si="4"/>
+        <v>1.4115708063811312</v>
+      </c>
+      <c r="G26">
+        <f t="shared" si="5"/>
+        <v>1.4115708063811312</v>
+      </c>
+      <c r="H26">
+        <f t="shared" si="6"/>
+        <v>1.4115708063811312</v>
+      </c>
+      <c r="I26">
+        <f t="shared" si="7"/>
+        <v>1.4115708063811312</v>
+      </c>
+      <c r="J26">
+        <f t="shared" si="8"/>
+        <v>1.4115708063811312</v>
+      </c>
+      <c r="K26">
+        <f t="shared" si="9"/>
+        <v>1.4115708063811312</v>
+      </c>
+      <c r="L26">
+        <f t="shared" si="10"/>
+        <v>14.115708063811311</v>
+      </c>
+      <c r="M26" s="9">
+        <v>10.287000000000001</v>
+      </c>
+      <c r="N26">
+        <v>470051.87199999986</v>
+      </c>
+      <c r="O26">
+        <v>645000</v>
+      </c>
+      <c r="P26">
+        <f t="shared" si="11"/>
+        <v>1.3721889825810547</v>
       </c>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B27" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C27" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D27" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E27" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F27" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G27" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H27" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I27" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J27" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K27" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L27" t="e">
-        <f t="shared" si="10"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P27" t="e">
-        <f t="shared" si="11"/>
-        <v>#DIV/0!</v>
+      <c r="B27">
+        <f t="shared" si="0"/>
+        <v>46.533105873335231</v>
+      </c>
+      <c r="C27">
+        <f t="shared" si="1"/>
+        <v>46.533105873335231</v>
+      </c>
+      <c r="D27">
+        <f t="shared" si="2"/>
+        <v>46.533105873335231</v>
+      </c>
+      <c r="E27">
+        <f t="shared" si="3"/>
+        <v>46.533105873335231</v>
+      </c>
+      <c r="F27">
+        <f t="shared" si="4"/>
+        <v>46.533105873335231</v>
+      </c>
+      <c r="G27">
+        <f t="shared" si="5"/>
+        <v>46.533105873335231</v>
+      </c>
+      <c r="H27">
+        <f t="shared" si="6"/>
+        <v>46.533105873335231</v>
+      </c>
+      <c r="I27">
+        <f t="shared" si="7"/>
+        <v>46.533105873335231</v>
+      </c>
+      <c r="J27">
+        <f t="shared" si="8"/>
+        <v>46.533105873335231</v>
+      </c>
+      <c r="K27">
+        <f t="shared" si="9"/>
+        <v>46.533105873335231</v>
+      </c>
+      <c r="L27">
+        <f t="shared" si="10"/>
+        <v>465.33105873335234</v>
+      </c>
+      <c r="M27" s="11">
+        <v>41.296999999999997</v>
+      </c>
+      <c r="N27">
+        <v>81647.763000000356</v>
+      </c>
+      <c r="O27">
+        <v>920000</v>
+      </c>
+      <c r="P27">
+        <f t="shared" si="11"/>
+        <v>11.267914345675289</v>
       </c>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B28" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C28" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D28" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E28" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F28" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G28" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H28" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I28" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J28" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K28" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L28" t="e">
-        <f t="shared" si="10"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P28" t="e">
-        <f t="shared" si="11"/>
-        <v>#DIV/0!</v>
+      <c r="B28">
+        <f t="shared" si="0"/>
+        <v>9.9593733928023624</v>
+      </c>
+      <c r="C28">
+        <f t="shared" si="1"/>
+        <v>9.9593733928023624</v>
+      </c>
+      <c r="D28">
+        <f t="shared" si="2"/>
+        <v>9.9593733928023624</v>
+      </c>
+      <c r="E28">
+        <f t="shared" si="3"/>
+        <v>9.9593733928023624</v>
+      </c>
+      <c r="F28">
+        <f t="shared" si="4"/>
+        <v>9.9593733928023624</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="5"/>
+        <v>9.9593733928023624</v>
+      </c>
+      <c r="H28">
+        <f t="shared" si="6"/>
+        <v>9.9593733928023624</v>
+      </c>
+      <c r="I28">
+        <f t="shared" si="7"/>
+        <v>9.9593733928023624</v>
+      </c>
+      <c r="J28">
+        <f t="shared" si="8"/>
+        <v>9.9593733928023624</v>
+      </c>
+      <c r="K28">
+        <f t="shared" si="9"/>
+        <v>9.9593733928023624</v>
+      </c>
+      <c r="L28">
+        <f t="shared" si="10"/>
+        <v>99.593733928023624</v>
+      </c>
+      <c r="M28" s="11">
+        <v>72.766999999999996</v>
+      </c>
+      <c r="N28">
+        <v>4383830.0139999986</v>
+      </c>
+      <c r="O28">
+        <v>6000000</v>
+      </c>
+      <c r="P28">
+        <f t="shared" si="11"/>
+        <v>1.3686662075944265</v>
       </c>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B29" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C29" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D29" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E29" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F29" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G29" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H29" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I29" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J29" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K29" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L29" t="e">
-        <f t="shared" si="10"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P29" t="e">
-        <f t="shared" si="11"/>
-        <v>#DIV/0!</v>
+      <c r="B29">
+        <f t="shared" si="0"/>
+        <v>1.9793729188243283E-3</v>
+      </c>
+      <c r="C29">
+        <f t="shared" si="1"/>
+        <v>1.9793729188243283E-3</v>
+      </c>
+      <c r="D29">
+        <f t="shared" si="2"/>
+        <v>1.9793729188243283E-3</v>
+      </c>
+      <c r="E29">
+        <f t="shared" si="3"/>
+        <v>1.9793729188243283E-3</v>
+      </c>
+      <c r="F29">
+        <f t="shared" si="4"/>
+        <v>1.9793729188243283E-3</v>
+      </c>
+      <c r="G29">
+        <f t="shared" si="5"/>
+        <v>1.9793729188243283E-3</v>
+      </c>
+      <c r="H29">
+        <f t="shared" si="6"/>
+        <v>1.9793729188243283E-3</v>
+      </c>
+      <c r="I29">
+        <f t="shared" si="7"/>
+        <v>1.9793729188243283E-3</v>
+      </c>
+      <c r="J29">
+        <f t="shared" si="8"/>
+        <v>1.9793729188243283E-3</v>
+      </c>
+      <c r="K29">
+        <f t="shared" si="9"/>
+        <v>1.9793729188243283E-3</v>
+      </c>
+      <c r="L29">
+        <f t="shared" si="10"/>
+        <v>1.9793729188243285E-2</v>
+      </c>
+      <c r="M29" s="12">
+        <v>1.0999999999999999E-2</v>
+      </c>
+      <c r="N29">
+        <v>1055889.9640000025</v>
+      </c>
+      <c r="O29">
+        <v>1900000</v>
+      </c>
+      <c r="P29">
+        <f t="shared" si="11"/>
+        <v>1.799429926203935</v>
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B30" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C30" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D30" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E30" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F30" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G30" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H30" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I30" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J30" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K30" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L30" t="e">
-        <f t="shared" si="10"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P30" t="e">
-        <f t="shared" si="11"/>
-        <v>#DIV/0!</v>
+      <c r="B30">
+        <f t="shared" si="0"/>
+        <v>25.993604122325753</v>
+      </c>
+      <c r="C30">
+        <f t="shared" si="1"/>
+        <v>25.993604122325753</v>
+      </c>
+      <c r="D30">
+        <f t="shared" si="2"/>
+        <v>25.993604122325753</v>
+      </c>
+      <c r="E30">
+        <f t="shared" si="3"/>
+        <v>25.993604122325753</v>
+      </c>
+      <c r="F30">
+        <f t="shared" si="4"/>
+        <v>25.993604122325753</v>
+      </c>
+      <c r="G30">
+        <f t="shared" si="5"/>
+        <v>25.993604122325753</v>
+      </c>
+      <c r="H30">
+        <f t="shared" si="6"/>
+        <v>25.993604122325753</v>
+      </c>
+      <c r="I30">
+        <f t="shared" si="7"/>
+        <v>25.993604122325753</v>
+      </c>
+      <c r="J30">
+        <f t="shared" si="8"/>
+        <v>25.993604122325753</v>
+      </c>
+      <c r="K30">
+        <f t="shared" si="9"/>
+        <v>25.993604122325753</v>
+      </c>
+      <c r="L30">
+        <f t="shared" si="10"/>
+        <v>259.93604122325752</v>
+      </c>
+      <c r="M30" s="9">
+        <v>130.489</v>
+      </c>
+      <c r="N30">
+        <v>5796141.185000075</v>
+      </c>
+      <c r="O30">
+        <v>11546000</v>
+      </c>
+      <c r="P30">
+        <f t="shared" si="11"/>
+        <v>1.9920149684897386</v>
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B31" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C31" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D31" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E31" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F31" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G31" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H31" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I31" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J31" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K31" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L31" t="e">
-        <f t="shared" si="10"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P31" t="e">
-        <f t="shared" si="11"/>
-        <v>#DIV/0!</v>
+      <c r="B31">
+        <f t="shared" si="0"/>
+        <v>1.1065993076178222</v>
+      </c>
+      <c r="C31">
+        <f t="shared" si="1"/>
+        <v>1.1065993076178222</v>
+      </c>
+      <c r="D31">
+        <f t="shared" si="2"/>
+        <v>1.1065993076178222</v>
+      </c>
+      <c r="E31">
+        <f t="shared" si="3"/>
+        <v>1.1065993076178222</v>
+      </c>
+      <c r="F31">
+        <f t="shared" si="4"/>
+        <v>1.1065993076178222</v>
+      </c>
+      <c r="G31">
+        <f t="shared" si="5"/>
+        <v>1.1065993076178222</v>
+      </c>
+      <c r="H31">
+        <f t="shared" si="6"/>
+        <v>1.1065993076178222</v>
+      </c>
+      <c r="I31">
+        <f t="shared" si="7"/>
+        <v>1.1065993076178222</v>
+      </c>
+      <c r="J31">
+        <f t="shared" si="8"/>
+        <v>1.1065993076178222</v>
+      </c>
+      <c r="K31">
+        <f t="shared" si="9"/>
+        <v>1.1065993076178222</v>
+      </c>
+      <c r="L31">
+        <f t="shared" si="10"/>
+        <v>11.065993076178222</v>
+      </c>
+      <c r="M31" s="9">
+        <v>4.5030000000000001</v>
+      </c>
+      <c r="N31">
+        <v>265720.30000000005</v>
+      </c>
+      <c r="O31">
+        <v>653000</v>
+      </c>
+      <c r="P31">
+        <f t="shared" si="11"/>
+        <v>2.4574712583118412</v>
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B32" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C32" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D32" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E32" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F32" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G32" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H32" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I32" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J32" t="e">
-        <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K32" t="e">
-        <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L32" t="e">
-        <f t="shared" si="10"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P32" t="e">
-        <f t="shared" si="11"/>
-        <v>#DIV/0!</v>
+      <c r="B32">
+        <f t="shared" si="0"/>
+        <v>0.36825801382039963</v>
+      </c>
+      <c r="C32">
+        <f t="shared" si="1"/>
+        <v>0.36825801382039963</v>
+      </c>
+      <c r="D32">
+        <f t="shared" si="2"/>
+        <v>0.36825801382039963</v>
+      </c>
+      <c r="E32">
+        <f t="shared" si="3"/>
+        <v>0.36825801382039963</v>
+      </c>
+      <c r="F32">
+        <f t="shared" si="4"/>
+        <v>0.36825801382039963</v>
+      </c>
+      <c r="G32">
+        <f t="shared" si="5"/>
+        <v>0.36825801382039963</v>
+      </c>
+      <c r="H32">
+        <f t="shared" si="6"/>
+        <v>0.36825801382039963</v>
+      </c>
+      <c r="I32">
+        <f t="shared" si="7"/>
+        <v>0.36825801382039963</v>
+      </c>
+      <c r="J32">
+        <f t="shared" si="8"/>
+        <v>0.36825801382039963</v>
+      </c>
+      <c r="K32">
+        <f t="shared" si="9"/>
+        <v>0.36825801382039963</v>
+      </c>
+      <c r="L32">
+        <f t="shared" si="10"/>
+        <v>3.6825801382039964</v>
+      </c>
+      <c r="M32" s="9">
+        <v>2.7490000000000001</v>
+      </c>
+      <c r="N32">
+        <v>1041350.0470000005</v>
+      </c>
+      <c r="O32">
+        <v>1395000</v>
+      </c>
+      <c r="P32">
+        <f t="shared" si="11"/>
+        <v>1.3396071801396858</v>
       </c>
     </row>
   </sheetData>

</xml_diff>